<commit_message>
Fix: ajusta base 100 do JMBI11 e adiciona trava de diversificacao na Opcao 4
</commit_message>
<xml_diff>
--- a/Dados/Simulacao_Oasis_Comparativa.xlsx
+++ b/Dados/Simulacao_Oasis_Comparativa.xlsx
@@ -446,10 +446,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45665.19887858592</v>
+        <v>45685.09514298425</v>
       </c>
       <c r="C2" t="n">
-        <v>459.9788785859184</v>
+        <v>458.6651429842485</v>
       </c>
       <c r="D2" t="n">
         <v>2500</v>
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48657.05975579425</v>
+        <v>48675.52134278624</v>
       </c>
       <c r="C3" t="n">
-        <v>491.860877208334</v>
+        <v>490.4261998019929</v>
       </c>
       <c r="D3" t="n">
         <v>2500</v>
@@ -478,10 +478,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51681.14603334435</v>
+        <v>51698.04955205909</v>
       </c>
       <c r="C4" t="n">
-        <v>524.0862775501042</v>
+        <v>522.5282092728526</v>
       </c>
       <c r="D4" t="n">
         <v>2500</v>
@@ -494,10 +494,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54737.80481174318</v>
+        <v>54753.02438355805</v>
       </c>
       <c r="C5" t="n">
-        <v>556.6587783988192</v>
+        <v>554.9748314989562</v>
       </c>
       <c r="D5" t="n">
         <v>2500</v>
@@ -510,10 +510,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57827.38693012497</v>
+        <v>57840.79414943141</v>
       </c>
       <c r="C6" t="n">
-        <v>589.5821183817931</v>
+        <v>587.7697658733645</v>
       </c>
       <c r="D6" t="n">
         <v>2500</v>
@@ -526,10 +526,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60950.24700652014</v>
+        <v>60961.71090093327</v>
       </c>
       <c r="C7" t="n">
-        <v>622.8600763951779</v>
+        <v>620.9167515018559</v>
       </c>
       <c r="D7" t="n">
         <v>2500</v>
@@ -542,10 +542,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64106.74347855784</v>
+        <v>64116.13046856251</v>
       </c>
       <c r="C8" t="n">
-        <v>656.496472037701</v>
+        <v>654.4195676292397</v>
       </c>
       <c r="D8" t="n">
         <v>2500</v>
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>67297.23864460691</v>
+        <v>67304.41250263275</v>
       </c>
       <c r="C9" t="n">
-        <v>690.4951660490726</v>
+        <v>688.2820340702453</v>
       </c>
       <c r="D9" t="n">
         <v>2500</v>
@@ -574,10 +574,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>70522.09870536003</v>
+        <v>70526.92051427779</v>
       </c>
       <c r="C10" t="n">
-        <v>724.8600607531168</v>
+        <v>722.5080116450378</v>
       </c>
       <c r="D10" t="n">
         <v>2500</v>
@@ -590,10 +590,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>73781.6938058657</v>
+        <v>73784.0219168972</v>
       </c>
       <c r="C11" t="n">
-        <v>759.5951005056748</v>
+        <v>757.101402619408</v>
       </c>
       <c r="D11" t="n">
         <v>2500</v>
@@ -606,10 +606,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>77076.39807801302</v>
+        <v>77076.08806804688</v>
       </c>
       <c r="C12" t="n">
-        <v>794.7042721473325</v>
+        <v>792.0661511496883</v>
       </c>
       <c r="D12" t="n">
         <v>2500</v>
@@ -622,10 +622,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>80406.58968347404</v>
+        <v>80403.49431177933</v>
       </c>
       <c r="C13" t="n">
-        <v>830.1916054610249</v>
+        <v>827.406243732445</v>
       </c>
       <c r="D13" t="n">
         <v>2500</v>
@@ -638,10 +638,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>83772.65085710862</v>
+        <v>83766.62002143833</v>
       </c>
       <c r="C14" t="n">
-        <v>866.0611736345689</v>
+        <v>863.1257096589974</v>
       </c>
       <c r="D14" t="n">
         <v>2500</v>
@@ -654,10 +654,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>87174.9679508368</v>
+        <v>87165.84864291314</v>
       </c>
       <c r="C15" t="n">
-        <v>902.3170937281789</v>
+        <v>899.2286214748159</v>
       </c>
       <c r="D15" t="n">
         <v>2500</v>
@@ -670,10 +670,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>90613.93147798382</v>
+        <v>90601.567738357</v>
       </c>
       <c r="C16" t="n">
-        <v>938.963527147016</v>
+        <v>935.7190954438532</v>
       </c>
       <c r="D16" t="n">
         <v>2500</v>
@@ -686,10 +686,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>94089.93615810265</v>
+        <v>94074.16903037486</v>
       </c>
       <c r="C17" t="n">
-        <v>976.0046801188298</v>
+        <v>972.6012920178583</v>
       </c>
       <c r="D17" t="n">
         <v>2500</v>
@@ -702,10 +702,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>97603.38096227939</v>
+        <v>97584.04844668559</v>
       </c>
       <c r="C18" t="n">
-        <v>1013.444804176743</v>
+        <v>1009.87941631073</v>
       </c>
       <c r="D18" t="n">
         <v>2500</v>
@@ -718,10 +718,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>101154.6691589266</v>
+        <v>101131.6061652635</v>
       </c>
       <c r="C19" t="n">
-        <v>1051.288196647236</v>
+        <v>1047.557718577959</v>
       </c>
       <c r="D19" t="n">
         <v>2500</v>
@@ -734,10 +734,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>104744.20836007</v>
+        <v>104717.2466599648</v>
       </c>
       <c r="C20" t="n">
-        <v>1089.539201143388</v>
+        <v>1085.640494701226</v>
       </c>
       <c r="D20" t="n">
         <v>2500</v>
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>108372.4105681334</v>
+        <v>108341.3787466429</v>
       </c>
       <c r="C21" t="n">
-        <v>1128.202208063436</v>
+        <v>1124.132086678188</v>
       </c>
       <c r="D21" t="n">
         <v>2500</v>
@@ -766,10 +766,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>112039.6922232281</v>
+        <v>112004.4156297605</v>
       </c>
       <c r="C22" t="n">
-        <v>1167.281655094688</v>
+        <v>1163.036883117536</v>
       </c>
       <c r="D22" t="n">
         <v>2500</v>
@@ -782,10 +782,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>115746.474250951</v>
+        <v>115706.7749494998</v>
       </c>
       <c r="C23" t="n">
-        <v>1206.782027722885</v>
+        <v>1202.359319739358</v>
       </c>
       <c r="D23" t="n">
         <v>2500</v>
@@ -798,10 +798,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>119493.1821106981</v>
+        <v>119448.8788293807</v>
       </c>
       <c r="C24" t="n">
-        <v>1246.707859747037</v>
+        <v>1242.103879880875</v>
       </c>
       <c r="D24" t="n">
         <v>2500</v>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>123280.2458444979</v>
+        <v>123231.1539243883</v>
       </c>
       <c r="C25" t="n">
-        <v>1287.063733799798</v>
+        <v>1282.275095007612</v>
       </c>
       <c r="D25" t="n">
         <v>2500</v>
@@ -830,10 +830,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>127108.1001263713</v>
+        <v>127054.0314696184</v>
       </c>
       <c r="C26" t="n">
-        <v>1327.854281873468</v>
+        <v>1322.877545230049</v>
       </c>
       <c r="D26" t="n">
         <v>2500</v>
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>130977.184312223</v>
+        <v>130917.9473294442</v>
       </c>
       <c r="C27" t="n">
-        <v>1369.084185851634</v>
+        <v>1363.91585982582</v>
       </c>
       <c r="D27" t="n">
         <v>2500</v>
@@ -862,10 +862,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>134887.9424902695</v>
+        <v>134823.3420472117</v>
       </c>
       <c r="C28" t="n">
-        <v>1410.758178046559</v>
+        <v>1405.394717767523</v>
       </c>
       <c r="D28" t="n">
         <v>2500</v>
@@ -878,10 +878,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>138840.8235320119</v>
+        <v>138770.6608954679</v>
       </c>
       <c r="C29" t="n">
-        <v>1452.881041742345</v>
+        <v>1447.318848256187</v>
       </c>
       <c r="D29" t="n">
         <v>2500</v>
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>142836.2811437558</v>
+        <v>142760.3539267284</v>
       </c>
       <c r="C30" t="n">
-        <v>1495.457611743956</v>
+        <v>1489.693031260474</v>
       </c>
       <c r="D30" t="n">
         <v>2500</v>
@@ -910,10 +910,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>146874.773918688</v>
+        <v>146792.87602479</v>
       </c>
       <c r="C31" t="n">
-        <v>1538.492774932146</v>
+        <v>1532.522098061663</v>
       </c>
       <c r="D31" t="n">
         <v>2500</v>
@@ -926,10 +926,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>150956.7653895124</v>
+        <v>150868.6869565946</v>
       </c>
       <c r="C32" t="n">
-        <v>1581.991470824372</v>
+        <v>1575.810931804492</v>
       </c>
       <c r="D32" t="n">
         <v>2500</v>
@@ -942,10 +942,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>155082.7240816541</v>
+        <v>154988.2514246484</v>
       </c>
       <c r="C33" t="n">
-        <v>1625.958692141745</v>
+        <v>1619.564468053901</v>
       </c>
       <c r="D33" t="n">
         <v>2500</v>
@@ -958,10 +958,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>159253.1235670362</v>
+        <v>159152.0391200062</v>
       </c>
       <c r="C34" t="n">
-        <v>1670.399485382084</v>
+        <v>1663.787695357769</v>
       </c>
       <c r="D34" t="n">
         <v>2500</v>
@@ -974,10 +974,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>163468.4425184353</v>
+        <v>163360.5247758219</v>
       </c>
       <c r="C35" t="n">
-        <v>1715.31895139915</v>
+        <v>1708.485655815671</v>
       </c>
       <c r="D35" t="n">
         <v>2500</v>
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>167729.1647644234</v>
+        <v>167614.1882214757</v>
       </c>
       <c r="C36" t="n">
-        <v>1760.722245988115</v>
+        <v>1753.663445653761</v>
       </c>
       <c r="D36" t="n">
         <v>2500</v>
@@ -1006,10 +1006,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>172035.7793449008</v>
+        <v>171913.5144372815</v>
       </c>
       <c r="C37" t="n">
-        <v>1806.614580477334</v>
+        <v>1799.326215805811</v>
       </c>
       <c r="D37" t="n">
         <v>2500</v>
@@ -1022,10 +1022,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>176388.7805672273</v>
+        <v>176258.993609782</v>
       </c>
       <c r="C38" t="n">
-        <v>1853.001222326497</v>
+        <v>1845.479172500496</v>
       </c>
       <c r="D38" t="n">
         <v>2500</v>
@@ -1038,10 +1038,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>180788.6680629585</v>
+        <v>180651.1211876369</v>
       </c>
       <c r="C39" t="n">
-        <v>1899.887495731221</v>
+        <v>1892.12757785498</v>
       </c>
       <c r="D39" t="n">
         <v>2500</v>
@@ -1054,10 +1054,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>185235.9468451926</v>
+        <v>185090.3979381118</v>
       </c>
       <c r="C40" t="n">
-        <v>1947.278782234151</v>
+        <v>1939.276750474877</v>
       </c>
       <c r="D40" t="n">
         <v>2500</v>
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>189731.1273665353</v>
+        <v>189577.3300041725</v>
       </c>
       <c r="C41" t="n">
-        <v>1995.180521342649</v>
+        <v>1986.932066060645</v>
       </c>
       <c r="D41" t="n">
         <v>2500</v>
@@ -1086,10 +1086,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>194274.7255776884</v>
+        <v>194112.428962193</v>
       </c>
       <c r="C42" t="n">
-        <v>2043.598211153132</v>
+        <v>2035.0989580205</v>
       </c>
       <c r="D42" t="n">
         <v>2500</v>
@@ -1102,10 +1102,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>198867.2629866705</v>
+        <v>198696.2118802829</v>
       </c>
       <c r="C43" t="n">
-        <v>2092.537408982138</v>
+        <v>2083.782918089904</v>
       </c>
       <c r="D43" t="n">
         <v>2500</v>
@@ -1118,10 +1118,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>203509.2667186747</v>
+        <v>203329.2013772406</v>
       </c>
       <c r="C44" t="n">
-        <v>2142.003732004182</v>
+        <v>2132.989496957702</v>
       </c>
       <c r="D44" t="n">
         <v>2500</v>
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>208201.2695765712</v>
+        <v>208011.9256821396</v>
       </c>
       <c r="C45" t="n">
-        <v>2192.002857896495</v>
+        <v>2182.724304898984</v>
       </c>
       <c r="D45" t="n">
         <v>2500</v>
@@ -1150,10 +1150,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>212943.8101020619</v>
+        <v>212744.9186945543</v>
       </c>
       <c r="C46" t="n">
-        <v>2242.540525490695</v>
+        <v>2232.993012414738</v>
       </c>
       <c r="D46" t="n">
         <v>2500</v>
@@ -1166,10 +1166,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>217737.4326374934</v>
+        <v>217528.7200454327</v>
       </c>
       <c r="C47" t="n">
-        <v>2293.622535431481</v>
+        <v>2283.801350878369</v>
       </c>
       <c r="D47" t="n">
         <v>2500</v>
@@ -1182,10 +1182,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>222582.6873883358</v>
+        <v>222363.8751586219</v>
       </c>
       <c r="C48" t="n">
-        <v>2345.25475084243</v>
+        <v>2335.155113189165</v>
       </c>
       <c r="D48" t="n">
         <v>2500</v>
@@ -1198,10 +1198,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>227480.1304863347</v>
+        <v>227250.9353130547</v>
       </c>
       <c r="C49" t="n">
-        <v>2397.443097998951</v>
+        <v>2387.060154432768</v>
       </c>
       <c r="D49" t="n">
         <v>2500</v>
@@ -1214,10 +1214,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>232430.3240533432</v>
+        <v>232190.4577056034</v>
       </c>
       <c r="C50" t="n">
-        <v>2450.193567008498</v>
+        <v>2439.522392548743</v>
       </c>
       <c r="D50" t="n">
         <v>2500</v>
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>237433.8362658414</v>
+        <v>237183.0055146087</v>
       </c>
       <c r="C51" t="n">
-        <v>2503.512212498108</v>
+        <v>2492.547809005308</v>
       </c>
       <c r="D51" t="n">
         <v>2500</v>
@@ -1246,10 +1246,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>242491.2414201507</v>
+        <v>242229.14796409</v>
       </c>
       <c r="C52" t="n">
-        <v>2557.405154309339</v>
+        <v>2546.142449481311</v>
       </c>
       <c r="D52" t="n">
         <v>2500</v>
@@ -1262,10 +1262,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>247603.1199983514</v>
+        <v>247329.4603886455</v>
       </c>
       <c r="C53" t="n">
-        <v>2611.878578200701</v>
+        <v>2600.312424555527</v>
       </c>
       <c r="D53" t="n">
         <v>2500</v>
@@ -1278,10 +1278,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>252770.058734909</v>
+        <v>252484.5242990489</v>
       </c>
       <c r="C54" t="n">
-        <v>2666.938736557645</v>
+        <v>2655.063910403353</v>
       </c>
       <c r="D54" t="n">
         <v>2500</v>
@@ -1294,10 +1294,10 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>257992.6506840193</v>
+        <v>257694.9274485499</v>
       </c>
       <c r="C55" t="n">
-        <v>2722.591949110207</v>
+        <v>2710.403149500981</v>
       </c>
       <c r="D55" t="n">
         <v>2500</v>
@@ -1310,10 +1310,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>263271.4952876776</v>
+        <v>262961.263899887</v>
       </c>
       <c r="C56" t="n">
-        <v>2778.844603658376</v>
+        <v>2766.336451337138</v>
       </c>
       <c r="D56" t="n">
         <v>2500</v>
@@ -1326,10 +1326,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>268607.1984444829</v>
+        <v>268284.1340930194</v>
       </c>
       <c r="C57" t="n">
-        <v>2835.703156805277</v>
+        <v>2822.870193132456</v>
       </c>
       <c r="D57" t="n">
         <v>2500</v>
@@ -1342,10 +1342,10 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>274000.3725791811</v>
+        <v>273664.144913586</v>
       </c>
       <c r="C58" t="n">
-        <v>2893.174134698252</v>
+        <v>2880.010820566568</v>
       </c>
       <c r="D58" t="n">
         <v>2500</v>
@@ -1358,10 +1358,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>279451.636712959</v>
+        <v>279101.909762099</v>
       </c>
       <c r="C59" t="n">
-        <v>2951.264133777921</v>
+        <v>2937.764848513016</v>
       </c>
       <c r="D59" t="n">
         <v>2500</v>
@@ -1374,10 +1374,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>284961.6165344943</v>
+        <v>284598.048623881</v>
       </c>
       <c r="C60" t="n">
-        <v>3009.979821535315</v>
+        <v>2996.138861782038</v>
       </c>
       <c r="D60" t="n">
         <v>2500</v>
@@ -1390,10 +1390,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>290530.9444717715</v>
+        <v>290153.1881397524</v>
       </c>
       <c r="C61" t="n">
-        <v>3069.327937277158</v>
+        <v>3055.139515871335</v>
       </c>
       <c r="D61" t="n">
         <v>2500</v>
@@ -1406,10 +1406,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>296160.2597646709</v>
+        <v>295767.9616774773</v>
       </c>
       <c r="C62" t="n">
-        <v>3129.315292899397</v>
+        <v>3114.773537724895</v>
       </c>
       <c r="D62" t="n">
         <v>2500</v>
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>301850.2085383399</v>
+        <v>301443.0094039773</v>
       </c>
       <c r="C63" t="n">
-        <v>3189.948773669064</v>
+        <v>3175.047726499964</v>
       </c>
       <c r="D63" t="n">
         <v>2500</v>
@@ -1438,10 +1438,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>307601.4438773545</v>
+        <v>307178.9783583195</v>
       </c>
       <c r="C64" t="n">
-        <v>3251.235339014557</v>
+        <v>3235.968954342251</v>
       </c>
       <c r="D64" t="n">
         <v>2500</v>
@@ -1454,10 +1454,10 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>313414.6259006789</v>
+        <v>312976.5225254889</v>
       </c>
       <c r="C65" t="n">
-        <v>3313.182023324428</v>
+        <v>3297.544167169454</v>
       </c>
       <c r="D65" t="n">
         <v>2500</v>
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>319290.4218374337</v>
+        <v>318836.3029109521</v>
       </c>
       <c r="C66" t="n">
-        <v>3375.795936754791</v>
+        <v>3359.780385463195</v>
       </c>
       <c r="D66" t="n">
         <v>2500</v>
@@ -1486,10 +1486,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>325229.5061034791</v>
+        <v>324758.9876160216</v>
       </c>
       <c r="C67" t="n">
-        <v>3439.084266045406</v>
+        <v>3422.684705069462</v>
       </c>
       <c r="D67" t="n">
         <v>2500</v>
@@ -1502,10 +1502,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>331232.5603788237</v>
+        <v>330745.2519140292</v>
       </c>
       <c r="C68" t="n">
-        <v>3503.05427534457</v>
+        <v>3486.264298007634</v>
       </c>
       <c r="D68" t="n">
         <v>2500</v>
@@ -1518,10 +1518,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>337300.2736858666</v>
+        <v>336795.7783273174</v>
       </c>
       <c r="C69" t="n">
-        <v>3567.713307042883</v>
+        <v>3550.526413288203</v>
       </c>
       <c r="D69" t="n">
         <v>2500</v>
@@ -1534,10 +1534,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>343433.3424684826</v>
+        <v>342911.2567050567</v>
       </c>
       <c r="C70" t="n">
-        <v>3633.068782615996</v>
+        <v>3615.478377739266</v>
       </c>
       <c r="D70" t="n">
         <v>2500</v>
@@ -1550,10 +1550,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>349632.470671959</v>
+        <v>349092.3843018986</v>
       </c>
       <c r="C71" t="n">
-        <v>3699.128203476444</v>
+        <v>3681.127596841888</v>
       </c>
       <c r="D71" t="n">
         <v>2500</v>
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>355898.3698237937</v>
+        <v>355339.8658574731</v>
       </c>
       <c r="C72" t="n">
-        <v>3765.899151834641</v>
+        <v>3747.481555574443</v>
       </c>
       <c r="D72" t="n">
         <v>2500</v>
@@ -1582,10 +1582,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>362231.7591153629</v>
+        <v>361654.413676739</v>
       </c>
       <c r="C73" t="n">
-        <v>3833.389291569159</v>
+        <v>3814.547819266003</v>
       </c>
       <c r="D73" t="n">
         <v>2500</v>
@@ -1598,10 +1598,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>368633.3654844693</v>
+        <v>368036.7477111979</v>
       </c>
       <c r="C74" t="n">
-        <v>3901.60636910638</v>
+        <v>3882.334034458906</v>
       </c>
       <c r="D74" t="n">
         <v>2500</v>
@@ -1614,10 +1614,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>375103.9236987789</v>
+        <v>374487.5956409785</v>
       </c>
       <c r="C75" t="n">
-        <v>3970.558214309614</v>
+        <v>3950.847929780568</v>
       </c>
       <c r="D75" t="n">
         <v>2500</v>
@@ -1630,10 +1630,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>381644.1764401567</v>
+        <v>381007.6929578031</v>
       </c>
       <c r="C76" t="n">
-        <v>4040.252741377804</v>
+        <v>4020.097316824664</v>
       </c>
       <c r="D76" t="n">
         <v>2500</v>
@@ -1646,10 +1646,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>388254.8743899106</v>
+        <v>387597.7830488449</v>
       </c>
       <c r="C77" t="n">
-        <v>4110.69794975391</v>
+        <v>4090.09009104176</v>
       </c>
       <c r="D77" t="n">
         <v>2500</v>
@@ -1662,10 +1662,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>394936.7763149537</v>
+        <v>394258.6172814844</v>
       </c>
       <c r="C78" t="n">
-        <v>4181.901925043067</v>
+        <v>4160.83423263952</v>
       </c>
       <c r="D78" t="n">
         <v>2500</v>
@@ -1678,10 +1678,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>401690.6491548943</v>
+        <v>400990.9550889769</v>
       </c>
       <c r="C79" t="n">
-        <v>4253.872839940647</v>
+        <v>4232.337807492555</v>
       </c>
       <c r="D79" t="n">
         <v>2500</v>
@@ -1694,10 +1694,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>408517.2681100647</v>
+        <v>407795.564057039</v>
       </c>
       <c r="C80" t="n">
-        <v>4326.618955170303</v>
+        <v>4304.608968062063</v>
       </c>
       <c r="D80" t="n">
         <v>2500</v>
@@ -1710,10 +1710,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>415417.4167304968</v>
+        <v>414673.2200113643</v>
       </c>
       <c r="C81" t="n">
-        <v>4400.148620432128</v>
+        <v>4377.655954325322</v>
       </c>
       <c r="D81" t="n">
         <v>2500</v>
@@ -1726,10 +1726,10 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>422391.8870058578</v>
+        <v>421624.7071060795</v>
       </c>
       <c r="C82" t="n">
-        <v>4474.470275361023</v>
+        <v>4451.487094715171</v>
       </c>
       <c r="D82" t="n">
         <v>2500</v>
@@ -1742,10 +1742,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>429441.4794563532</v>
+        <v>428650.8179131491</v>
       </c>
       <c r="C83" t="n">
-        <v>4549.592450495384</v>
+        <v>4526.110807069578</v>
       </c>
       <c r="D83" t="n">
         <v>2500</v>
@@ -1758,10 +1758,10 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>436567.0032246095</v>
+        <v>435752.3535127405</v>
       </c>
       <c r="C84" t="n">
-        <v>4625.523768256225</v>
+        <v>4601.535599591391</v>
       </c>
       <c r="D84" t="n">
         <v>2500</v>
@@ -1774,10 +1774,10 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>443769.2761685463</v>
+        <v>442930.1235845588</v>
       </c>
       <c r="C85" t="n">
-        <v>4702.272943936851</v>
+        <v>4677.770071818401</v>
       </c>
       <c r="D85" t="n">
         <v>2500</v>
@@ -1790,10 +1790,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>451049.1249552495</v>
+        <v>450184.9465001627</v>
       </c>
       <c r="C86" t="n">
-        <v>4779.848786703187</v>
+        <v>4754.82291560382</v>
       </c>
       <c r="D86" t="n">
         <v>2500</v>
@@ -1806,10 +1806,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>458407.3851558544</v>
+        <v>457517.6494162699</v>
       </c>
       <c r="C87" t="n">
-        <v>4858.260200604879</v>
+        <v>4832.702916107274</v>
       </c>
       <c r="D87" t="n">
         <v>2500</v>
@@ -1822,10 +1822,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>465844.9013414517</v>
+        <v>464929.0683690663</v>
       </c>
       <c r="C88" t="n">
-        <v>4937.51618559729</v>
+        <v>4911.418952796447</v>
       </c>
       <c r="D88" t="n">
         <v>2500</v>
@@ -1838,10 +1838,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>473362.5271800262</v>
+        <v>472420.0483695258</v>
       </c>
       <c r="C89" t="n">
-        <v>5017.625838574506</v>
+        <v>4990.980000459464</v>
       </c>
       <c r="D89" t="n">
         <v>2500</v>
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>480961.1255344396</v>
+        <v>479991.443499754</v>
       </c>
       <c r="C90" t="n">
-        <v>5098.59835441346</v>
+        <v>5071.395130228155</v>
       </c>
       <c r="D90" t="n">
         <v>2500</v>
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>488641.568561469</v>
+        <v>487644.1170103662</v>
       </c>
       <c r="C91" t="n">
-        <v>5180.443027029311</v>
+        <v>5152.673510612294</v>
       </c>
       <c r="D91" t="n">
         <v>2500</v>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>496404.7378119112</v>
+        <v>495378.9414189112</v>
       </c>
       <c r="C92" t="n">
-        <v>5263.169250442186</v>
+        <v>5234.82440854495</v>
       </c>
       <c r="D92" t="n">
         <v>2500</v>
@@ -1902,10 +1902,10 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>504251.5243317666</v>
+        <v>503196.7986093502</v>
       </c>
       <c r="C93" t="n">
-        <v>5346.786519855413</v>
+        <v>5317.857190439045</v>
       </c>
       <c r="D93" t="n">
         <v>2500</v>
@@ -1918,10 +1918,10 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>512182.828764512</v>
+        <v>511098.5799326055</v>
       </c>
       <c r="C94" t="n">
-        <v>5431.304432745364</v>
+        <v>5401.781323255271</v>
       </c>
       <c r="D94" t="n">
         <v>2500</v>
@@ -1934,10 +1934,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>520199.561454475</v>
+        <v>519085.186308187</v>
       </c>
       <c r="C95" t="n">
-        <v>5516.732689963047</v>
+        <v>5486.606375581458</v>
       </c>
       <c r="D95" t="n">
         <v>2500</v>
@@ -1950,10 +1950,10 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>528302.6425513226</v>
+        <v>527157.5283269105</v>
       </c>
       <c r="C96" t="n">
-        <v>5603.081096847552</v>
+        <v>5572.342018723535</v>
       </c>
       <c r="D96" t="n">
         <v>2500</v>
@@ -1966,10 +1966,10 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>536493.0021156741</v>
+        <v>535316.5263547186</v>
       </c>
       <c r="C97" t="n">
-        <v>5690.359564351494</v>
+        <v>5658.998027808207</v>
       </c>
       <c r="D97" t="n">
         <v>2500</v>
@@ -1982,10 +1982,10 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>544771.5802258527</v>
+        <v>543563.110637616</v>
       </c>
       <c r="C98" t="n">
-        <v>5778.578110178581</v>
+        <v>5746.584282897453</v>
       </c>
       <c r="D98" t="n">
         <v>2500</v>
@@ -1998,10 +1998,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>553139.3270857861</v>
+        <v>551898.2214077311</v>
       </c>
       <c r="C99" t="n">
-        <v>5867.746859933432</v>
+        <v>5835.110770115009</v>
       </c>
       <c r="D99" t="n">
         <v>2500</v>
@@ -2014,10 +2014,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>561597.2031340699</v>
+        <v>560322.808990516</v>
       </c>
       <c r="C100" t="n">
-        <v>5957.87604828378</v>
+        <v>5924.587582784927</v>
       </c>
       <c r="D100" t="n">
         <v>2500</v>
@@ -2030,10 +2030,10 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>570146.1791542051</v>
+        <v>568837.8339130983</v>
       </c>
       <c r="C101" t="n">
-        <v>6048.97602013519</v>
+        <v>6015.024922582363</v>
       </c>
       <c r="D101" t="n">
         <v>2500</v>
@@ -2046,10 +2046,10 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>578787.2363860236</v>
+        <v>577444.2670137951</v>
       </c>
       <c r="C102" t="n">
-        <v>6141.057231818439</v>
+        <v>6106.433100696721</v>
       </c>
       <c r="D102" t="n">
         <v>2500</v>
@@ -2062,10 +2062,10 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>587521.3666383133</v>
+        <v>586143.0895528024</v>
       </c>
       <c r="C103" t="n">
-        <v>6234.130252289674</v>
+        <v>6198.822539007281</v>
       </c>
       <c r="D103" t="n">
         <v>2500</v>
@@ -2078,10 +2078,10 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>596349.5724026568</v>
+        <v>594935.2933240738</v>
       </c>
       <c r="C104" t="n">
-        <v>6328.205764343506</v>
+        <v>6292.203771271441</v>
       </c>
       <c r="D104" t="n">
         <v>2500</v>
@@ -2094,10 +2094,10 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>605272.8669684959</v>
+        <v>603821.8807683995</v>
       </c>
       <c r="C105" t="n">
-        <v>6423.294565839165</v>
+        <v>6386.587444325727</v>
       </c>
       <c r="D105" t="n">
         <v>2500</v>
@@ -2110,10 +2110,10 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>614292.2745394357</v>
+        <v>612803.8650876991</v>
       </c>
       <c r="C106" t="n">
-        <v>6519.407570939865</v>
+        <v>6481.984319299688</v>
       </c>
       <c r="D106" t="n">
         <v>2500</v>
@@ -2126,10 +2126,10 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>623408.8303508012</v>
+        <v>621882.270360542</v>
       </c>
       <c r="C107" t="n">
-        <v>6616.555811365514</v>
+        <v>6578.40527284282</v>
       </c>
       <c r="D107" t="n">
         <v>2500</v>
@@ -2142,10 +2142,10 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>632623.5807884602</v>
+        <v>631058.1316589067</v>
       </c>
       <c r="C108" t="n">
-        <v>6714.750437658924</v>
+        <v>6675.861298364666</v>
       </c>
       <c r="D108" t="n">
         <v>2500</v>
@@ -2158,10 +2158,10 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>641937.5835089259</v>
+        <v>640332.495166195</v>
       </c>
       <c r="C109" t="n">
-        <v>6814.002720465651</v>
+        <v>6774.363507288232</v>
       </c>
       <c r="D109" t="n">
         <v>2500</v>
@@ -2174,10 +2174,10 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>651351.9075607535</v>
+        <v>649706.4182965119</v>
       </c>
       <c r="C110" t="n">
-        <v>6914.324051827624</v>
+        <v>6873.923130316842</v>
       </c>
       <c r="D110" t="n">
         <v>2500</v>
@@ -2190,10 +2190,10 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>660867.6335072443</v>
+        <v>659180.9698152265</v>
       </c>
       <c r="C111" t="n">
-        <v>7015.725946490715</v>
+        <v>6974.551518714612</v>
       </c>
       <c r="D111" t="n">
         <v>2500</v>
@@ -2242,10 +2242,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45596.20204679803</v>
+        <v>45616.29537153661</v>
       </c>
       <c r="C2" t="n">
-        <v>390.9820467980306</v>
+        <v>389.8653715366112</v>
       </c>
       <c r="D2" t="n">
         <v>2500</v>
@@ -2258,10 +2258,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48513.65210097112</v>
+        <v>48532.52986487359</v>
       </c>
       <c r="C3" t="n">
-        <v>417.4500541730882</v>
+        <v>416.2344933369794</v>
       </c>
       <c r="D3" t="n">
         <v>2500</v>
@@ -2274,10 +2274,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51457.81248689316</v>
+        <v>51475.37409003775</v>
       </c>
       <c r="C4" t="n">
-        <v>444.1603859220317</v>
+        <v>442.8442251641576</v>
       </c>
       <c r="D4" t="n">
         <v>2500</v>
@@ -2290,10 +2290,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54428.92774750708</v>
+        <v>54445.07085254748</v>
       </c>
       <c r="C5" t="n">
-        <v>471.115260613919</v>
+        <v>469.6967625097303</v>
       </c>
       <c r="D5" t="n">
         <v>2500</v>
@@ -2306,10 +2306,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57427.2446646367</v>
+        <v>57441.86517344594</v>
       </c>
       <c r="C6" t="n">
-        <v>498.3169171296258</v>
+        <v>496.794320898459</v>
       </c>
       <c r="D6" t="n">
         <v>2500</v>
@@ -2322,10 +2322,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60453.01227948451</v>
+        <v>60466.00430951702</v>
       </c>
       <c r="C7" t="n">
-        <v>525.7676148478088</v>
+        <v>524.139136071079</v>
       </c>
       <c r="D7" t="n">
         <v>2500</v>
@@ -2338,10 +2338,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>63506.48191331707</v>
+        <v>63517.73777368578</v>
       </c>
       <c r="C8" t="n">
-        <v>553.4696338325697</v>
+        <v>551.7334641687636</v>
       </c>
       <c r="D8" t="n">
         <v>2500</v>
@@ -2354,10 +2354,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>66587.90718833992</v>
+        <v>66597.31735560506</v>
       </c>
       <c r="C9" t="n">
-        <v>581.4252750228385</v>
+        <v>579.5795819192722</v>
       </c>
       <c r="D9" t="n">
         <v>2500</v>
@@ -2370,10 +2370,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>69697.5440487634</v>
+        <v>69704.99714242986</v>
       </c>
       <c r="C10" t="n">
-        <v>609.63686042349</v>
+        <v>607.679786824796</v>
       </c>
       <c r="D10" t="n">
         <v>2500</v>
@@ -2386,10 +2386,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>72835.65078206161</v>
+        <v>72841.03353978138</v>
       </c>
       <c r="C11" t="n">
-        <v>638.1067332982108</v>
+        <v>636.0363973515184</v>
       </c>
       <c r="D11" t="n">
         <v>2500</v>
@@ -2402,10 +2402,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>76002.48804042574</v>
+        <v>76005.68529290229</v>
       </c>
       <c r="C12" t="n">
-        <v>666.8372583641304</v>
+        <v>664.6517531209048</v>
       </c>
       <c r="D12" t="n">
         <v>2500</v>
@@ -2418,10 +2418,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>79198.31886241397</v>
+        <v>79199.21350800502</v>
       </c>
       <c r="C13" t="n">
-        <v>695.8308219882371</v>
+        <v>693.5282151027384</v>
       </c>
       <c r="D13" t="n">
         <v>2500</v>
@@ -2434,10 +2434,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>82423.40869479957</v>
+        <v>82421.88167381493</v>
       </c>
       <c r="C14" t="n">
-        <v>725.0898323855887</v>
+        <v>722.6681658099161</v>
       </c>
       <c r="D14" t="n">
         <v>2500</v>
@@ -2450,10 +2450,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>85678.02541461891</v>
+        <v>85673.95568330996</v>
       </c>
       <c r="C15" t="n">
-        <v>754.6167198193413</v>
+        <v>752.0740094950237</v>
       </c>
       <c r="D15" t="n">
         <v>2500</v>
@@ -2466,10 +2466,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>88962.43935142152</v>
+        <v>88955.70385565866</v>
       </c>
       <c r="C16" t="n">
-        <v>784.413936802606</v>
+        <v>781.7481723487032</v>
       </c>
       <c r="D16" t="n">
         <v>2500</v>
@@ -2482,10 +2482,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>92276.92330972367</v>
+        <v>92267.3969583585</v>
       </c>
       <c r="C17" t="n">
-        <v>814.4839583021572</v>
+        <v>811.6931026998305</v>
       </c>
       <c r="D17" t="n">
         <v>2500</v>
@@ -2498,10 +2498,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>95621.75259166767</v>
+        <v>95609.30822957603</v>
       </c>
       <c r="C18" t="n">
-        <v>844.8292819440027</v>
+        <v>841.9112712175209</v>
       </c>
       <c r="D18" t="n">
         <v>2500</v>
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>98997.20501988851</v>
+        <v>98981.71340069101</v>
       </c>
       <c r="C19" t="n">
-        <v>875.4524282208384</v>
+        <v>872.4051711149757</v>
       </c>
       <c r="D19" t="n">
         <v>2500</v>
@@ -2530,10 +2530,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>102403.5609605899</v>
+        <v>102384.8907190462</v>
       </c>
       <c r="C20" t="n">
-        <v>906.355940701401</v>
+        <v>903.1773183551906</v>
       </c>
       <c r="D20" t="n">
         <v>2500</v>
@@ -2546,10 +2546,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>105841.1033468316</v>
+        <v>105819.1209709047</v>
       </c>
       <c r="C21" t="n">
-        <v>937.5423862417368</v>
+        <v>934.23025185854</v>
       </c>
       <c r="D21" t="n">
         <v>2500</v>
@@ -2562,10 +2562,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>109310.1177020301</v>
+        <v>109284.687504617</v>
       </c>
       <c r="C22" t="n">
-        <v>969.0143551984073</v>
+        <v>965.5665337122566</v>
       </c>
       <c r="D22" t="n">
         <v>2500</v>
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>112810.8921636737</v>
+        <v>112781.8762539988</v>
       </c>
       <c r="C23" t="n">
-        <v>1000.774461643643</v>
+        <v>997.1887493818218</v>
       </c>
       <c r="D23" t="n">
         <v>2500</v>
@@ -2594,10 +2594,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>116343.7175072562</v>
+        <v>116310.9757619231</v>
       </c>
       <c r="C24" t="n">
-        <v>1032.825343582472</v>
+        <v>1029.099507924284</v>
       </c>
       <c r="D24" t="n">
         <v>2500</v>
@@ -2610,10 +2610,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>119908.887170428</v>
+        <v>119872.2772041266</v>
       </c>
       <c r="C25" t="n">
-        <v>1065.16966317183</v>
+        <v>1061.301442203524</v>
       </c>
       <c r="D25" t="n">
         <v>2500</v>
@@ -2626,10 +2626,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>123506.6972773697</v>
+        <v>123466.0744132341</v>
       </c>
       <c r="C26" t="n">
-        <v>1097.810106941682</v>
+        <v>1093.797209107488</v>
       </c>
       <c r="D26" t="n">
         <v>2500</v>
@@ -2642,10 +2642,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>127137.4466633879</v>
+        <v>127092.6639030015</v>
       </c>
       <c r="C27" t="n">
-        <v>1130.749386018167</v>
+        <v>1126.589489767397</v>
       </c>
       <c r="D27" t="n">
         <v>2500</v>
@@ -2658,10 +2658,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>130801.4368997366</v>
+        <v>130752.3448927805</v>
       </c>
       <c r="C28" t="n">
-        <v>1163.990236348784</v>
+        <v>1159.680989778957</v>
       </c>
       <c r="D28" t="n">
         <v>2500</v>
@@ -2674,10 +2674,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>134498.9723186663</v>
+        <v>134445.4193322061</v>
       </c>
       <c r="C29" t="n">
-        <v>1197.535418929641</v>
+        <v>1193.074439425596</v>
       </c>
       <c r="D29" t="n">
         <v>2500</v>
@@ -2690,10 +2690,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>138230.3600387011</v>
+        <v>138172.1919261098</v>
       </c>
       <c r="C30" t="n">
-        <v>1231.387720034783</v>
+        <v>1226.772593903727</v>
       </c>
       <c r="D30" t="n">
         <v>2500</v>
@@ -2706,10 +2706,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>141995.9099901487</v>
+        <v>141932.9701596599</v>
       </c>
       <c r="C31" t="n">
-        <v>1265.549951447623</v>
+        <v>1260.778233550071</v>
       </c>
       <c r="D31" t="n">
         <v>2500</v>
@@ -2722,10 +2722,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>145795.9349408432</v>
+        <v>145728.0643237309</v>
       </c>
       <c r="C32" t="n">
-        <v>1300.024950694488</v>
+        <v>1295.094164071057</v>
       </c>
       <c r="D32" t="n">
         <v>2500</v>
@@ -2738,10 +2738,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>149630.7505221235</v>
+        <v>149557.7875405053</v>
       </c>
       <c r="C33" t="n">
-        <v>1334.815581280307</v>
+        <v>1329.723216774314</v>
       </c>
       <c r="D33" t="n">
         <v>2500</v>
@@ -2754,10 +2754,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>153500.6752550499</v>
+        <v>153422.4557893075</v>
       </c>
       <c r="C34" t="n">
-        <v>1369.924732926451</v>
+        <v>1364.668248802267</v>
       </c>
       <c r="D34" t="n">
         <v>2500</v>
@@ -2770,10 +2770,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>157406.0305768607</v>
+        <v>157322.3879326754</v>
       </c>
       <c r="C35" t="n">
-        <v>1405.355321810758</v>
+        <v>1399.93214336788</v>
       </c>
       <c r="D35" t="n">
         <v>2500</v>
@@ -2786,10 +2786,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>161347.1408676704</v>
+        <v>161257.905742668</v>
       </c>
       <c r="C36" t="n">
-        <v>1441.110290809751</v>
+        <v>1435.517809992536</v>
       </c>
       <c r="D36" t="n">
         <v>2500</v>
@@ -2802,10 +2802,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>165324.3334774135</v>
+        <v>165229.3339274141</v>
       </c>
       <c r="C37" t="n">
-        <v>1477.19260974307</v>
+        <v>1471.428184746095</v>
       </c>
       <c r="D37" t="n">
         <v>2500</v>
@@ -2818,10 +2818,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>169337.9387530336</v>
+        <v>169237.0001579032</v>
       </c>
       <c r="C38" t="n">
-        <v>1513.605275620154</v>
+        <v>1507.666230489139</v>
       </c>
       <c r="D38" t="n">
         <v>2500</v>
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>173388.2900659228</v>
+        <v>173281.2350950206</v>
       </c>
       <c r="C39" t="n">
-        <v>1550.351312889165</v>
+        <v>1544.234937117434</v>
       </c>
       <c r="D39" t="n">
         <v>2500</v>
@@ -2850,10 +2850,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>177475.723839611</v>
+        <v>177362.3724168293</v>
       </c>
       <c r="C40" t="n">
-        <v>1587.433773688208</v>
+        <v>1581.137321808611</v>
       </c>
       <c r="D40" t="n">
         <v>2500</v>
@@ -2866,10 +2866,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>181600.5795777099</v>
+        <v>181480.7488461004</v>
       </c>
       <c r="C41" t="n">
-        <v>1624.855738098836</v>
+        <v>1618.376429271108</v>
       </c>
       <c r="D41" t="n">
         <v>2500</v>
@@ -2882,10 +2882,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>185763.1998921118</v>
+        <v>185636.7041780957</v>
       </c>
       <c r="C42" t="n">
-        <v>1662.620314401885</v>
+        <v>1655.955331995379</v>
       </c>
       <c r="D42" t="n">
         <v>2500</v>
@@ -2898,10 +2898,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>189963.9305314474</v>
+        <v>189830.5813086031</v>
       </c>
       <c r="C43" t="n">
-        <v>1700.730639335649</v>
+        <v>1693.8771305074</v>
       </c>
       <c r="D43" t="n">
         <v>2500</v>
@@ -2914,10 +2914,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>194203.1204098038</v>
+        <v>194062.7262622276</v>
       </c>
       <c r="C44" t="n">
-        <v>1739.189878356421</v>
+        <v>1732.144953624477</v>
       </c>
       <c r="D44" t="n">
         <v>2500</v>
@@ -2930,10 +2930,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>198481.1216357052</v>
+        <v>198333.488220941</v>
       </c>
       <c r="C45" t="n">
-        <v>1778.001225901412</v>
+        <v>1770.761958713402</v>
       </c>
       <c r="D45" t="n">
         <v>2500</v>
@@ -2946,10 +2946,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>202798.2895413593</v>
+        <v>202643.219552892</v>
       </c>
       <c r="C46" t="n">
-        <v>1817.167905654084</v>
+        <v>1809.731331950956</v>
       </c>
       <c r="D46" t="n">
         <v>2500</v>
@@ -2962,10 +2962,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>207154.9827121712</v>
+        <v>206992.2758414788</v>
       </c>
       <c r="C47" t="n">
-        <v>1856.693170811913</v>
+        <v>1849.056288586791</v>
       </c>
       <c r="D47" t="n">
         <v>2500</v>
@@ -2978,10 +2978,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>211551.5630165278</v>
+        <v>211381.0159146875</v>
       </c>
       <c r="C48" t="n">
-        <v>1896.580304356595</v>
+        <v>1888.74007320871</v>
       </c>
       <c r="D48" t="n">
         <v>2500</v>
@@ -2994,10 +2994,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>215988.3956358546</v>
+        <v>215809.8018746978</v>
       </c>
       <c r="C49" t="n">
-        <v>1936.832619326738</v>
+        <v>1928.785960010372</v>
       </c>
       <c r="D49" t="n">
         <v>2500</v>
@@ -3010,10 +3010,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>220465.8490949476</v>
+        <v>220278.9991277593</v>
       </c>
       <c r="C50" t="n">
-        <v>1977.453459093039</v>
+        <v>1969.197253061431</v>
       </c>
       <c r="D50" t="n">
         <v>2500</v>
@@ -3026,10 +3026,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>224984.2952925836</v>
+        <v>224788.9764143394</v>
       </c>
       <c r="C51" t="n">
-        <v>2018.446197635988</v>
+        <v>2009.97728658015</v>
       </c>
       <c r="D51" t="n">
         <v>2500</v>
@@ -3042,10 +3042,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>229544.1095324097</v>
+        <v>229340.1058395479</v>
       </c>
       <c r="C52" t="n">
-        <v>2059.814239826112</v>
+        <v>2051.129425208494</v>
       </c>
       <c r="D52" t="n">
         <v>2500</v>
@@ -3058,10 +3058,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>234145.6705541165</v>
+        <v>233932.7629038377</v>
       </c>
       <c r="C53" t="n">
-        <v>2101.561021706782</v>
+        <v>2092.65706428974</v>
       </c>
       <c r="D53" t="n">
         <v>2500</v>
@@ -3074,10 +3074,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>238789.3605648961</v>
+        <v>238567.3265339863</v>
       </c>
       <c r="C54" t="n">
-        <v>2143.690010779615</v>
+        <v>2134.563630148614</v>
       </c>
       <c r="D54" t="n">
         <v>2500</v>
@@ -3090,10 +3090,10 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>243475.5652711886</v>
+        <v>243244.1791143603</v>
       </c>
       <c r="C55" t="n">
-        <v>2186.204706292487</v>
+        <v>2176.852580373989</v>
       </c>
       <c r="D55" t="n">
         <v>2500</v>
@@ -3106,10 +3106,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>248204.6739107188</v>
+        <v>247963.7065184644</v>
       </c>
       <c r="C56" t="n">
-        <v>2229.108639530175</v>
+        <v>2219.527404104159</v>
       </c>
       <c r="D56" t="n">
         <v>2500</v>
@@ -3122,10 +3122,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>252977.0792848264</v>
+        <v>252726.2981407791</v>
       </c>
       <c r="C57" t="n">
-        <v>2272.405374107675</v>
+        <v>2262.591622314721</v>
       </c>
       <c r="D57" t="n">
         <v>2500</v>
@@ -3138,10 +3138,10 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>257793.1777910926</v>
+        <v>257532.3469288882</v>
       </c>
       <c r="C58" t="n">
-        <v>2316.098506266192</v>
+        <v>2306.048788109075</v>
       </c>
       <c r="D58" t="n">
         <v>2500</v>
@@ -3154,10 +3154,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>262653.3694562645</v>
+        <v>262382.2494158998</v>
       </c>
       <c r="C59" t="n">
-        <v>2360.191665171846</v>
+        <v>2349.902487011586</v>
       </c>
       <c r="D59" t="n">
         <v>2500</v>
@@ -3170,10 +3170,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>267558.0579694816</v>
+        <v>267276.4057531632</v>
       </c>
       <c r="C60" t="n">
-        <v>2404.688513217111</v>
+        <v>2394.156337263412</v>
       </c>
       <c r="D60" t="n">
         <v>2500</v>
@@ -3186,10 +3186,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>272507.6507158066</v>
+        <v>272215.2197432842</v>
       </c>
       <c r="C61" t="n">
-        <v>2449.592746325017</v>
+        <v>2438.813990121033</v>
       </c>
       <c r="D61" t="n">
         <v>2500</v>
@@ -3202,10 +3202,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>277502.5588100627</v>
+        <v>277199.0988734417</v>
       </c>
       <c r="C62" t="n">
-        <v>2494.908094256132</v>
+        <v>2483.87913015751</v>
       </c>
       <c r="D62" t="n">
         <v>2500</v>
@@ -3218,10 +3218,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>282543.1971309811</v>
+        <v>282228.4543490082</v>
       </c>
       <c r="C63" t="n">
-        <v>2540.63832091836</v>
+        <v>2529.355475566486</v>
       </c>
       <c r="D63" t="n">
         <v>2500</v>
@@ -3234,10 +3234,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>287629.9843556606</v>
+        <v>287303.7011274772</v>
       </c>
       <c r="C64" t="n">
-        <v>2586.787224679569</v>
+        <v>2575.246778468962</v>
       </c>
       <c r="D64" t="n">
         <v>2500</v>
@@ -3250,10 +3250,10 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>292763.3429943437</v>
+        <v>292425.2579527</v>
       </c>
       <c r="C65" t="n">
-        <v>2633.358638683087</v>
+        <v>2621.556825222875</v>
       </c>
       <c r="D65" t="n">
         <v>2500</v>
@@ -3266,10 +3266,10 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>297943.6994255098</v>
+        <v>297593.5473894355</v>
       </c>
       <c r="C66" t="n">
-        <v>2680.356431166082</v>
+        <v>2668.2894367355</v>
       </c>
       <c r="D66" t="n">
         <v>2500</v>
@@ -3282,10 +3282,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>303171.4839312906</v>
+        <v>302808.9958582142</v>
       </c>
       <c r="C67" t="n">
-        <v>2727.784505780863</v>
+        <v>2715.448468778702</v>
       </c>
       <c r="D67" t="n">
         <v>2500</v>
@@ -3298,10 +3298,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>308447.1307332097</v>
+        <v>308072.0336705213</v>
       </c>
       <c r="C68" t="n">
-        <v>2775.646801919116</v>
+        <v>2763.037812307062</v>
       </c>
       <c r="D68" t="n">
         <v>2500</v>
@@ -3314,10 +3314,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>313771.0780282489</v>
+        <v>313383.0950643002</v>
       </c>
       <c r="C69" t="n">
-        <v>2823.94729503911</v>
+        <v>2811.061393778913</v>
       </c>
       <c r="D69" t="n">
         <v>2500</v>
@@ -3330,10 +3330,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>319143.7680252448</v>
+        <v>318742.6182397805</v>
       </c>
       <c r="C70" t="n">
-        <v>2872.689996995901</v>
+        <v>2859.523175480295</v>
       </c>
       <c r="D70" t="n">
         <v>2500</v>
@@ -3346,10 +3346,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>324565.6469816193</v>
+        <v>324151.0453956323</v>
       </c>
       <c r="C71" t="n">
-        <v>2921.878956374562</v>
+        <v>2908.427155851875</v>
       </c>
       <c r="D71" t="n">
         <v>2500</v>
@@ -3362,10 +3362,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>330037.1652404458</v>
+        <v>329608.8227654512</v>
       </c>
       <c r="C72" t="n">
-        <v>2971.518258826452</v>
+        <v>2957.777369818848</v>
       </c>
       <c r="D72" t="n">
         <v>2500</v>
@@ -3378,10 +3378,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>335558.7772678543</v>
+        <v>335116.400654575</v>
       </c>
       <c r="C73" t="n">
-        <v>3021.612027408577</v>
+        <v>3007.577889123843</v>
       </c>
       <c r="D73" t="n">
         <v>2500</v>
@@ -3394,10 +3394,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>341130.9416907803</v>
+        <v>340674.2334772379</v>
       </c>
       <c r="C74" t="n">
-        <v>3072.164422926053</v>
+        <v>3057.832822662875</v>
       </c>
       <c r="D74" t="n">
         <v>2500</v>
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>346754.1213350581</v>
+        <v>346282.7797940622</v>
       </c>
       <c r="C75" t="n">
-        <v>3123.1796442777</v>
+        <v>3108.546316824354</v>
       </c>
       <c r="D75" t="n">
         <v>2500</v>
@@ -3426,10 +3426,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>352428.7832638629</v>
+        <v>351942.5023498934</v>
       </c>
       <c r="C76" t="n">
-        <v>3174.661928804808</v>
+        <v>3159.722555831193</v>
       </c>
       <c r="D76" t="n">
         <v>2500</v>
@@ -3442,10 +3442,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>358155.398816506</v>
+        <v>357653.8681119794</v>
       </c>
       <c r="C77" t="n">
-        <v>3226.615552643088</v>
+        <v>3211.36576208604</v>
       </c>
       <c r="D77" t="n">
         <v>2500</v>
@@ -3458,10 +3458,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>363934.4436475838</v>
+        <v>363417.3483084991</v>
       </c>
       <c r="C78" t="n">
-        <v>3279.044831077851</v>
+        <v>3263.480196519648</v>
       </c>
       <c r="D78" t="n">
         <v>2500</v>
@@ -3474,10 +3474,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>369766.3977664863</v>
+        <v>369233.4184674415</v>
       </c>
       <c r="C79" t="n">
-        <v>3331.95411890244</v>
+        <v>3316.07015894244</v>
       </c>
       <c r="D79" t="n">
         <v>2500</v>
@@ -3490,10 +3490,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>375651.7455772662</v>
+        <v>375102.5584558408</v>
       </c>
       <c r="C80" t="n">
-        <v>3385.347810779936</v>
+        <v>3369.139988399268</v>
       </c>
       <c r="D80" t="n">
         <v>2500</v>
@@ -3506,10 +3506,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>381590.9759188744</v>
+        <v>381025.2525193682</v>
       </c>
       <c r="C81" t="n">
-        <v>3439.230341608183</v>
+        <v>3422.694063527418</v>
       </c>
       <c r="D81" t="n">
         <v>2500</v>
@@ -3522,10 +3522,10 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>387584.5821057625</v>
+        <v>387001.9893222861</v>
       </c>
       <c r="C82" t="n">
-        <v>3493.606186888149</v>
+        <v>3476.73680291788</v>
       </c>
       <c r="D82" t="n">
         <v>2500</v>
@@ -3538,10 +3538,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>393633.0619688582</v>
+        <v>393033.261987766</v>
       </c>
       <c r="C83" t="n">
-        <v>3548.479863095668</v>
+        <v>3531.272665479908</v>
       </c>
       <c r="D83" t="n">
         <v>2500</v>
@@ -3554,10 +3554,10 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>399736.9178969148</v>
+        <v>399119.5681385749</v>
       </c>
       <c r="C84" t="n">
-        <v>3603.855928056575</v>
+        <v>3586.306150808917</v>
       </c>
       <c r="D84" t="n">
         <v>2500</v>
@@ -3570,10 +3570,10 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>405896.6568782401</v>
+        <v>405261.4099381327</v>
       </c>
       <c r="C85" t="n">
-        <v>3659.738981325282</v>
+        <v>3641.841799557729</v>
       </c>
       <c r="D85" t="n">
         <v>2500</v>
@@ -3586,10 +3586,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>412112.7905428068</v>
+        <v>411459.2941319439</v>
       </c>
       <c r="C86" t="n">
-        <v>3716.133664566819</v>
+        <v>3697.884193811207</v>
       </c>
       <c r="D86" t="n">
         <v>2500</v>
@@ -3602,10 +3602,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>418385.8352047492</v>
+        <v>417713.7320894082</v>
       </c>
       <c r="C87" t="n">
-        <v>3773.044661942374</v>
+        <v>3754.437957464316</v>
       </c>
       <c r="D87" t="n">
         <v>2500</v>
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>424716.3119052476</v>
+        <v>424025.2398460119</v>
       </c>
       <c r="C88" t="n">
-        <v>3830.476700498356</v>
+        <v>3811.50775660362</v>
       </c>
       <c r="D88" t="n">
         <v>2500</v>
@@ -3634,10 +3634,10 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>431104.7464558066</v>
+        <v>430394.3381459041</v>
       </c>
       <c r="C89" t="n">
-        <v>3888.43455055903</v>
+        <v>3869.09829989227</v>
       </c>
       <c r="D89" t="n">
         <v>2500</v>
@@ -3650,10 +3650,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>437551.6694819293</v>
+        <v>436821.5524848626</v>
       </c>
       <c r="C90" t="n">
-        <v>3946.923026122739</v>
+        <v>3927.214338958504</v>
       </c>
       <c r="D90" t="n">
         <v>2500</v>
@@ -3666,10 +3666,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>444057.6164671911</v>
+        <v>443307.4131536503</v>
       </c>
       <c r="C91" t="n">
-        <v>4005.946985261758</v>
+        <v>3985.860668787686</v>
       </c>
       <c r="D91" t="n">
         <v>2500</v>
@@ -3682,10 +3682,10 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>450623.1277977169</v>
+        <v>449852.4552817682</v>
       </c>
       <c r="C92" t="n">
-        <v>4065.511330525806</v>
+        <v>4045.042128117932</v>
       </c>
       <c r="D92" t="n">
         <v>2500</v>
@@ -3698,10 +3698,10 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>457248.7488070661</v>
+        <v>456457.2188816076</v>
       </c>
       <c r="C93" t="n">
-        <v>4125.621009349253</v>
+        <v>4104.763599839334</v>
       </c>
       <c r="D93" t="n">
         <v>2500</v>
@@ -3714,10 +3714,10 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>463935.0298215282</v>
+        <v>463122.2488930044</v>
       </c>
       <c r="C94" t="n">
-        <v>4186.281014462056</v>
+        <v>4165.030011396838</v>
       </c>
       <c r="D94" t="n">
         <v>2500</v>
@@ -3730,10 +3730,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>470682.5262058327</v>
+        <v>469848.0952282012</v>
       </c>
       <c r="C95" t="n">
-        <v>4247.496384304459</v>
+        <v>4225.846335196788</v>
       </c>
       <c r="D95" t="n">
         <v>2500</v>
@@ -3746,10 +3746,10 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>477491.7984092782</v>
+        <v>476635.3128172184</v>
       </c>
       <c r="C96" t="n">
-        <v>4309.272203445484</v>
+        <v>4287.21758901719</v>
       </c>
       <c r="D96" t="n">
         <v>2500</v>
@@ -3762,10 +3762,10 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>484363.4120122834</v>
+        <v>483484.4616536401</v>
       </c>
       <c r="C97" t="n">
-        <v>4371.613603005258</v>
+        <v>4349.148836421713</v>
       </c>
       <c r="D97" t="n">
         <v>2500</v>
@@ -3778,10 +3778,10 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>491297.9377733646</v>
+        <v>490396.1068408176</v>
       </c>
       <c r="C98" t="n">
-        <v>4434.525761081207</v>
+        <v>4411.645187177465</v>
       </c>
       <c r="D98" t="n">
         <v>2500</v>
@@ -3794,10 +3794,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>498295.9516765428</v>
+        <v>497370.8186384942</v>
       </c>
       <c r="C99" t="n">
-        <v>4498.013903178149</v>
+        <v>4474.711797676591</v>
       </c>
       <c r="D99" t="n">
         <v>2500</v>
@@ -3810,10 +3810,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>505358.0349791851</v>
+        <v>504409.1725098559</v>
       </c>
       <c r="C100" t="n">
-        <v>4562.083302642329</v>
+        <v>4538.353871361707</v>
       </c>
       <c r="D100" t="n">
         <v>2500</v>
@@ -3826,10 +3826,10 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>512484.7742602845</v>
+        <v>511511.7491690111</v>
       </c>
       <c r="C101" t="n">
-        <v>4626.73928109942</v>
+        <v>4602.576659155225</v>
       </c>
       <c r="D101" t="n">
         <v>2500</v>
@@ -3842,10 +3842,10 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>519676.761469181</v>
+        <v>518679.1346289037</v>
       </c>
       <c r="C102" t="n">
-        <v>4691.98720889654</v>
+        <v>4667.385459892586</v>
       </c>
       <c r="D102" t="n">
         <v>2500</v>
@@ -3858,10 +3858,10 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>526934.5939747294</v>
+        <v>525911.9202496632</v>
       </c>
       <c r="C103" t="n">
-        <v>4757.832505548323</v>
+        <v>4732.785620759458</v>
       </c>
       <c r="D103" t="n">
         <v>2500</v>
@@ -3874,10 +3874,10 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>534258.8746149165</v>
+        <v>533210.702787396</v>
       </c>
       <c r="C104" t="n">
-        <v>4824.280640187053</v>
+        <v>4798.782537732911</v>
       </c>
       <c r="D104" t="n">
         <v>2500</v>
@@ -3890,10 +3890,10 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>541650.2117469334</v>
+        <v>540576.0844434226</v>
       </c>
       <c r="C105" t="n">
-        <v>4891.33713201694</v>
+        <v>4865.381656026626</v>
       </c>
       <c r="D105" t="n">
         <v>2500</v>
@@ -3906,10 +3906,10 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>549109.2192977059</v>
+        <v>548008.6729139627</v>
       </c>
       <c r="C106" t="n">
-        <v>4959.007550772545</v>
+        <v>4932.588470540166</v>
       </c>
       <c r="D106" t="n">
         <v>2500</v>
@@ -3922,10 +3922,10 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>556636.5168148873</v>
+        <v>555509.0814402751</v>
       </c>
       <c r="C107" t="n">
-        <v>5027.297517181406</v>
+        <v>5000.408526312339</v>
       </c>
       <c r="D107" t="n">
         <v>2500</v>
@@ -3938,10 +3938,10 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>564232.7295183182</v>
+        <v>563077.9288592538</v>
       </c>
       <c r="C108" t="n">
-        <v>5096.212703430892</v>
+        <v>5068.847418978708</v>
       </c>
       <c r="D108" t="n">
         <v>2500</v>
@@ -3954,10 +3954,10 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>571898.4883519575</v>
+        <v>570715.839654487</v>
       </c>
       <c r="C109" t="n">
-        <v>5165.758833639346</v>
+        <v>5137.910795233266</v>
       </c>
       <c r="D109" t="n">
         <v>2500</v>
@@ -3970,10 +3970,10 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>579634.430036289</v>
+        <v>578423.4440077813</v>
       </c>
       <c r="C110" t="n">
-        <v>5235.941684331518</v>
+        <v>5207.604353294333</v>
       </c>
       <c r="D110" t="n">
         <v>2500</v>
@@ -3986,10 +3986,10 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>587441.1971212074</v>
+        <v>586201.3778511561</v>
       </c>
       <c r="C111" t="n">
-        <v>5306.767084918381</v>
+        <v>5277.933843374695</v>
       </c>
       <c r="D111" t="n">
         <v>2500</v>

</xml_diff>